<commit_message>
Record approved Phase 3 execution and regression fixes
</commit_message>
<xml_diff>
--- a/test-management/TEST_CASES.xlsx
+++ b/test-management/TEST_CASES.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" r:id="Rc334169345974f2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" r:id="R98658bfd0db14f90"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -132,7 +132,7 @@
         <x:color rgb="FF8F1C14"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE4E2"/>
         </x:patternFill>
       </x:fill>
@@ -143,7 +143,7 @@
         <x:color rgb="FF8A4B08"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1D6"/>
         </x:patternFill>
       </x:fill>
@@ -478,7 +478,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N2" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O2" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -527,7 +527,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N3" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O3" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -576,7 +576,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N4" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O4" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -624,7 +624,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N5" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O5" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -672,7 +672,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N6" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O6" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -720,7 +720,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N7" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O7" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -768,7 +768,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="N8" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O8" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -818,7 +818,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N9" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O9" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -866,7 +866,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N10" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O10" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -914,7 +914,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N11" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O11" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -963,7 +963,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N12" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O12" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -1011,7 +1011,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N13" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O13" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -1059,7 +1059,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N14" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O14" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -1109,7 +1109,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N15" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O15" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -1157,7 +1157,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N16" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O16" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -1205,7 +1205,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N17" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O17" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -1254,7 +1254,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="N18" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O18" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -1304,7 +1304,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N19" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O19" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -1352,7 +1352,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N20" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O20" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -1399,7 +1399,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N21" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O21" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -1446,7 +1446,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N22" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O22" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -1494,7 +1494,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N23" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O23" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -1542,7 +1542,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N24" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O24" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -1591,7 +1591,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N25" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O25" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -1640,7 +1640,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N26" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O26" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -1689,7 +1689,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N27" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O27" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -1738,7 +1738,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="N28" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O28" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -1786,7 +1786,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="N29" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O29" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -1836,7 +1836,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N30" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O30" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -1885,7 +1885,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N31" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O31" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -1935,7 +1935,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="N32" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O32" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -1985,7 +1985,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="N33" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O33" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -2034,7 +2034,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="N34" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O34" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -2082,7 +2082,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="N35" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O35" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -2131,7 +2131,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N36" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O36" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -2182,7 +2182,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="N37" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O37" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -2231,7 +2231,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="N38" s="3" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O38" s="3" t="str">
         <x:v>v1.0</x:v>
@@ -2255,7 +2255,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67db23dc610c4955"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4e0d80247ea43a1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Complete Phase 10 performance testing
</commit_message>
<xml_diff>
--- a/test-management/TEST_CASES.xlsx
+++ b/test-management/TEST_CASES.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" r:id="Raa64dce9467d4dd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" r:id="R2704479babab428d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2727,13 +2727,13 @@
         <x:v>The result reports all required measures without presenting local observations as production capacity.</x:v>
       </x:c>
       <x:c r="L49" s="8" t="str">
-        <x:v>release; performance; planned</x:v>
+        <x:v>release; performance; local-baseline</x:v>
       </x:c>
       <x:c r="M49" s="8" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="N49" s="8" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="O49" s="8" t="str">
         <x:v>v1.0</x:v>
@@ -2800,7 +2800,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bd22aaf949d4821"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R569ce891e7a24d4c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Complete Phase 11 simulated UAT
</commit_message>
<xml_diff>
--- a/test-management/TEST_CASES.xlsx
+++ b/test-management/TEST_CASES.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" r:id="R2704479babab428d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" r:id="R208cd96eea3a4194"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -138,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TestCasesTable" displayName="TestCasesTable" ref="A1:O50" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:O50"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TestCasesTable" displayName="TestCasesTable" ref="A1:O56" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:O56"/>
   <x:tableColumns count="15">
     <x:tableColumn id="1" name="Test Case ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -2786,21 +2786,303 @@
         <x:v>v1.0</x:v>
       </x:c>
     </x:row>
+    <x:row r="51" ht="36" hidden="0" customHeight="1">
+      <x:c r="A51" s="8" t="str">
+        <x:v>TC-UAT-001</x:v>
+      </x:c>
+      <x:c r="B51" s="8" t="str">
+        <x:v>Start a personal workspace</x:v>
+      </x:c>
+      <x:c r="C51" s="8" t="str">
+        <x:v>Confirm a new member can enter and understand the personal workspace.</x:v>
+      </x:c>
+      <x:c r="D51" s="8" t="str">
+        <x:v>UAT</x:v>
+      </x:c>
+      <x:c r="E51" s="8" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="F51" s="8" t="str">
+        <x:v>FR-AUTH-001; FR-PROFILE-001</x:v>
+      </x:c>
+      <x:c r="G51" s="8" t="str">
+        <x:v>AC-US001-01; AC-US005-01</x:v>
+      </x:c>
+      <x:c r="H51" s="8" t="str">
+        <x:v>Corrected local baseline is available; visitor is signed out.</x:v>
+      </x:c>
+      <x:c r="I51" s="8" t="str">
+        <x:v>UAT-MEMBER-A</x:v>
+      </x:c>
+      <x:c r="J51" s="8" t="str">
+        <x:v>1. Present the goal of starting a personal workspace. 2. Let the participant register without control-by-control coaching. 3. Ask the participant to identify their name and role.</x:v>
+      </x:c>
+      <x:c r="K51" s="8" t="str">
+        <x:v>The member workspace opens and the displayed identity and role are understandable.</x:v>
+      </x:c>
+      <x:c r="L51" s="8" t="str">
+        <x:v>uat; simulated; business-acceptance</x:v>
+      </x:c>
+      <x:c r="M51" s="8" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="N51" s="8" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="O51" s="8" t="str">
+        <x:v>v1.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="36" hidden="0" customHeight="1">
+      <x:c r="A52" s="16" t="str">
+        <x:v>TC-UAT-002</x:v>
+      </x:c>
+      <x:c r="B52" s="16" t="str">
+        <x:v>Maintain profile and daily work</x:v>
+      </x:c>
+      <x:c r="C52" s="16" t="str">
+        <x:v>Confirm the normal profile and personal-task lifecycle supports the participant's business goal.</x:v>
+      </x:c>
+      <x:c r="D52" s="16" t="str">
+        <x:v>UAT</x:v>
+      </x:c>
+      <x:c r="E52" s="16" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="F52" s="16" t="str">
+        <x:v>FR-PROFILE-001; FR-TASK-001; FR-TASK-003; FR-TASK-004; FR-TASK-005</x:v>
+      </x:c>
+      <x:c r="G52" s="16" t="str">
+        <x:v>AC-US003-01; AC-US003-04; AC-US003-05; AC-US003-06; AC-US003-07; AC-US003-08; AC-US003-09; AC-US005-02; AC-US005-03</x:v>
+      </x:c>
+      <x:c r="H52" s="16" t="str">
+        <x:v>UAT-MEMBER-A is signed in.</x:v>
+      </x:c>
+      <x:c r="I52" s="16" t="str">
+        <x:v>UAT-TASK-DAILY</x:v>
+      </x:c>
+      <x:c r="J52" s="16" t="str">
+        <x:v>1. Ask the participant to update their display name. 2. Ask them to create, revise, complete, reopen, cancel deletion, and then confirm deletion of daily work. 3. Observe feedback and questions.</x:v>
+      </x:c>
+      <x:c r="K52" s="16" t="str">
+        <x:v>Every intended change persists with clear feedback; canceled deletion preserves the task and confirmed deletion removes it.</x:v>
+      </x:c>
+      <x:c r="L52" s="16" t="str">
+        <x:v>uat; simulated; business-acceptance; lifecycle</x:v>
+      </x:c>
+      <x:c r="M52" s="16" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="N52" s="16" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="O52" s="16" t="str">
+        <x:v>v1.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="36" hidden="0" customHeight="1">
+      <x:c r="A53" s="8" t="str">
+        <x:v>TC-UAT-003</x:v>
+      </x:c>
+      <x:c r="B53" s="8" t="str">
+        <x:v>Find work that needs attention</x:v>
+      </x:c>
+      <x:c r="C53" s="8" t="str">
+        <x:v>Confirm search and state filters help the participant locate relevant personal work.</x:v>
+      </x:c>
+      <x:c r="D53" s="8" t="str">
+        <x:v>UAT</x:v>
+      </x:c>
+      <x:c r="E53" s="8" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="F53" s="8" t="str">
+        <x:v>FR-TASK-006</x:v>
+      </x:c>
+      <x:c r="G53" s="8" t="str">
+        <x:v>AC-US004-01; AC-US004-03; AC-US004-04; AC-US004-05; AC-US004-06</x:v>
+      </x:c>
+      <x:c r="H53" s="8" t="str">
+        <x:v>UAT-MEMBER-A owns active, completed, matching, and nonmatching tasks.</x:v>
+      </x:c>
+      <x:c r="I53" s="8" t="str">
+        <x:v>UAT-TASK-ACTIVE; UAT-TASK-COMPLETE; UAT-TASK-OTHER</x:v>
+      </x:c>
+      <x:c r="J53" s="8" t="str">
+        <x:v>1. Ask the participant to find work matching a business term. 2. Ask them to narrow the result by active and completed state. 3. Ask them to restore the complete list.</x:v>
+      </x:c>
+      <x:c r="K53" s="8" t="str">
+        <x:v>Every result satisfies both selected conditions and All restores the complete personal list.</x:v>
+      </x:c>
+      <x:c r="L53" s="8" t="str">
+        <x:v>uat; simulated; business-acceptance; search</x:v>
+      </x:c>
+      <x:c r="M53" s="8" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="N53" s="8" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="O53" s="8" t="str">
+        <x:v>v1.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="36" hidden="0" customHeight="1">
+      <x:c r="A54" s="16" t="str">
+        <x:v>TC-UAT-004</x:v>
+      </x:c>
+      <x:c r="B54" s="16" t="str">
+        <x:v>Continue after refreshing</x:v>
+      </x:c>
+      <x:c r="C54" s="16" t="str">
+        <x:v>Confirm a routine page refresh preserves a valid work session without repeating an action.</x:v>
+      </x:c>
+      <x:c r="D54" s="16" t="str">
+        <x:v>UAT</x:v>
+      </x:c>
+      <x:c r="E54" s="16" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="F54" s="16" t="str">
+        <x:v>NFR-REL-001</x:v>
+      </x:c>
+      <x:c r="G54" s="16" t="str">
+        <x:v>AC-US002-04; AC-US009-01</x:v>
+      </x:c>
+      <x:c r="H54" s="16" t="str">
+        <x:v>UAT-MEMBER-A is signed in and owns one uniquely named refresh task.</x:v>
+      </x:c>
+      <x:c r="I54" s="16" t="str">
+        <x:v>UAT-TASK-REFRESH</x:v>
+      </x:c>
+      <x:c r="J54" s="16" t="str">
+        <x:v>1. Ask the participant to refresh the authenticated workspace. 2. Ask them to confirm their identity and review the uniquely named task. 3. Count matching work items.</x:v>
+      </x:c>
+      <x:c r="K54" s="16" t="str">
+        <x:v>The member remains signed in and exactly one matching task is present after refresh.</x:v>
+      </x:c>
+      <x:c r="L54" s="16" t="str">
+        <x:v>uat; simulated; business-acceptance; continuity</x:v>
+      </x:c>
+      <x:c r="M54" s="16" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="N54" s="16" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="O54" s="16" t="str">
+        <x:v>v1.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="36" hidden="0" customHeight="1">
+      <x:c r="A55" s="8" t="str">
+        <x:v>TC-UAT-005</x:v>
+      </x:c>
+      <x:c r="B55" s="8" t="str">
+        <x:v>Review team workload</x:v>
+      </x:c>
+      <x:c r="C55" s="8" t="str">
+        <x:v>Confirm the administrator can understand team ownership and the read-only oversight boundary.</x:v>
+      </x:c>
+      <x:c r="D55" s="8" t="str">
+        <x:v>UAT</x:v>
+      </x:c>
+      <x:c r="E55" s="8" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="F55" s="8" t="str">
+        <x:v>FR-ADMIN-001; FR-ADMIN-002</x:v>
+      </x:c>
+      <x:c r="G55" s="8" t="str">
+        <x:v>AC-US006-01; AC-US006-02; AC-US006-05</x:v>
+      </x:c>
+      <x:c r="H55" s="8" t="str">
+        <x:v>UAT-MEMBER-B owns UAT-TASK-TEAM; UAT-ADMIN is signed in.</x:v>
+      </x:c>
+      <x:c r="I55" s="8" t="str">
+        <x:v>UAT-MEMBER-B; UAT-ADMIN; UAT-TASK-TEAM</x:v>
+      </x:c>
+      <x:c r="J55" s="8" t="str">
+        <x:v>1. Ask the participant to review team work and identify its owner. 2. Ask what actions are available for another member's task. 3. Record expectations before clarifying scope.</x:v>
+      </x:c>
+      <x:c r="K55" s="8" t="str">
+        <x:v>The owner is identifiable, no mutation actions are available for another member's task, and personal work remains separate.</x:v>
+      </x:c>
+      <x:c r="L55" s="8" t="str">
+        <x:v>uat; simulated; business-acceptance; admin</x:v>
+      </x:c>
+      <x:c r="M55" s="8" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="N55" s="8" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="O55" s="8" t="str">
+        <x:v>v1.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="24" hidden="0" customHeight="1">
+      <x:c r="A56" s="16" t="str">
+        <x:v>TC-UAT-006</x:v>
+      </x:c>
+      <x:c r="B56" s="16" t="str">
+        <x:v>Finish the work session</x:v>
+      </x:c>
+      <x:c r="C56" s="16" t="str">
+        <x:v>Confirm the participant can end the session and remain signed out after refresh.</x:v>
+      </x:c>
+      <x:c r="D56" s="16" t="str">
+        <x:v>UAT</x:v>
+      </x:c>
+      <x:c r="E56" s="16" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="F56" s="16" t="str">
+        <x:v>FR-AUTH-003</x:v>
+      </x:c>
+      <x:c r="G56" s="16" t="str">
+        <x:v>AC-US002-01</x:v>
+      </x:c>
+      <x:c r="H56" s="16" t="str">
+        <x:v>UAT-MEMBER-A is signed in.</x:v>
+      </x:c>
+      <x:c r="I56" s="16" t="str">
+        <x:v>UAT-MEMBER-A</x:v>
+      </x:c>
+      <x:c r="J56" s="16" t="str">
+        <x:v>1. Ask the participant to end the current session. 2. Ask them to refresh the resulting page. 3. Observe whether the workspace reopens.</x:v>
+      </x:c>
+      <x:c r="K56" s="16" t="str">
+        <x:v>The sign-in page remains displayed and the authenticated workspace does not reopen.</x:v>
+      </x:c>
+      <x:c r="L56" s="16" t="str">
+        <x:v>uat; simulated; business-acceptance; session</x:v>
+      </x:c>
+      <x:c r="M56" s="16" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="N56" s="16" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="O56" s="16" t="str">
+        <x:v>v1.0</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="3">
-    <x:dataValidation type="list" sqref="E2:E50">
+    <x:dataValidation type="list" sqref="E2:E56">
       <x:formula1>"Critical,High,Medium,Low"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="M2:M50">
+    <x:dataValidation type="list" sqref="M2:M56">
       <x:formula1>"Yes,Partial,No"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="N2:N50">
+    <x:dataValidation type="list" sqref="N2:N56">
       <x:formula1>"Approved,Draft,Retired"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R569ce891e7a24d4c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43d8ba200ac4419c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>